<commit_message>
data tranfer to new mac
</commit_message>
<xml_diff>
--- a/Pravartiya/data/test.xlsx
+++ b/Pravartiya/data/test.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="265" uniqueCount="10">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="137" uniqueCount="10">
   <si>
     <t>Verticals</t>
   </si>
@@ -51,7 +51,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" mc:Ignorable="x14ac">
   <numFmts count="0"/>
-  <fonts count="5" x14ac:knownFonts="1">
+  <fonts count="4" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -68,18 +68,12 @@
     </font>
     <font>
       <sz val="11"/>
-      <color theme="1"/>
+      <color rgb="FF000000"/>
       <name val="Calibri"/>
       <family val="2"/>
     </font>
     <font>
       <u/>
-      <sz val="11"/>
-      <color rgb="FF000000"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-    </font>
-    <font>
       <sz val="11"/>
       <color rgb="FF000000"/>
       <name val="Calibri"/>
@@ -128,7 +122,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="11">
+  <cellXfs count="12">
     <xf xfId="0" numFmtId="0" borderId="0" fontId="0" fillId="0"/>
     <xf xfId="0" numFmtId="0" borderId="1" applyBorder="1" fontId="1" applyFont="1" fillId="0" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -145,10 +139,13 @@
     <xf xfId="0" numFmtId="0" borderId="2" applyBorder="1" fontId="3" applyFont="1" fillId="0" quotePrefix="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf xfId="0" numFmtId="3" applyNumberFormat="1" borderId="2" applyBorder="1" fontId="4" applyFont="1" fillId="0" applyAlignment="1">
-      <alignment horizontal="right"/>
+    <xf xfId="0" numFmtId="0" borderId="0" fontId="0" fillId="0" applyAlignment="1">
+      <alignment horizontal="general"/>
     </xf>
-    <xf xfId="0" numFmtId="0" borderId="2" applyBorder="1" fontId="2" applyFont="1" fillId="0" quotePrefix="1" applyAlignment="1">
+    <xf xfId="0" numFmtId="0" borderId="2" applyBorder="1" fontId="3" applyFont="1" fillId="0" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf xfId="0" numFmtId="0" borderId="2" applyBorder="1" fontId="2" applyFont="1" fillId="0" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
     <xf xfId="0" numFmtId="0" borderId="0" fontId="0" fillId="0" applyAlignment="1">
@@ -465,15 +462,15 @@
   <dimension ref="A1:I33"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" style="8" width="12.43357142857143" customWidth="1" bestFit="1"/>
-    <col min="2" max="2" style="8" width="12.43357142857143" customWidth="1" bestFit="1"/>
-    <col min="3" max="3" style="9" width="12.43357142857143" customWidth="1" bestFit="1"/>
-    <col min="4" max="4" style="8" width="12.43357142857143" customWidth="1" bestFit="1"/>
-    <col min="5" max="5" style="8" width="12.43357142857143" customWidth="1" bestFit="1"/>
-    <col min="6" max="6" style="8" width="12.43357142857143" customWidth="1" bestFit="1"/>
-    <col min="7" max="7" style="10" width="12.43357142857143" customWidth="1" bestFit="1"/>
-    <col min="8" max="8" style="8" width="12.43357142857143" customWidth="1" bestFit="1"/>
-    <col min="9" max="9" style="8" width="12.43357142857143" customWidth="1" bestFit="1"/>
+    <col min="1" max="1" style="9" width="12.43357142857143" customWidth="1" bestFit="1"/>
+    <col min="2" max="2" style="9" width="12.43357142857143" customWidth="1" bestFit="1"/>
+    <col min="3" max="3" style="10" width="12.43357142857143" customWidth="1" bestFit="1"/>
+    <col min="4" max="4" style="9" width="12.43357142857143" customWidth="1" bestFit="1"/>
+    <col min="5" max="5" style="9" width="12.43357142857143" customWidth="1" bestFit="1"/>
+    <col min="6" max="6" style="9" width="12.43357142857143" customWidth="1" bestFit="1"/>
+    <col min="7" max="7" style="11" width="12.43357142857143" customWidth="1" bestFit="1"/>
+    <col min="8" max="8" style="9" width="12.43357142857143" customWidth="1" bestFit="1"/>
+    <col min="9" max="9" style="9" width="12.43357142857143" customWidth="1" bestFit="1"/>
   </cols>
   <sheetData>
     <row x14ac:dyDescent="0.25" r="1" customHeight="1" ht="20.25">
@@ -938,436 +935,180 @@
       </c>
     </row>
     <row x14ac:dyDescent="0.25" r="18" customHeight="1" ht="19.5">
-      <c r="A18" s="3" t="s">
-        <v>9</v>
-      </c>
-      <c r="B18" s="3" t="s">
-        <v>9</v>
-      </c>
+      <c r="A18" s="6"/>
+      <c r="B18" s="6"/>
       <c r="C18" s="4"/>
-      <c r="D18" s="3" t="s">
-        <v>9</v>
-      </c>
-      <c r="E18" s="3" t="s">
-        <v>9</v>
-      </c>
-      <c r="F18" s="3" t="s">
-        <v>9</v>
-      </c>
-      <c r="G18" s="5" t="s">
-        <v>9</v>
-      </c>
-      <c r="H18" s="3" t="s">
-        <v>9</v>
-      </c>
-      <c r="I18" s="3" t="s">
-        <v>9</v>
-      </c>
+      <c r="D18" s="6"/>
+      <c r="E18" s="6"/>
+      <c r="F18" s="6"/>
+      <c r="G18" s="7"/>
+      <c r="H18" s="6"/>
+      <c r="I18" s="6"/>
     </row>
     <row x14ac:dyDescent="0.25" r="19" customHeight="1" ht="19.5">
-      <c r="A19" s="3" t="s">
-        <v>9</v>
-      </c>
-      <c r="B19" s="3" t="s">
-        <v>9</v>
-      </c>
+      <c r="A19" s="6"/>
+      <c r="B19" s="6"/>
       <c r="C19" s="4"/>
-      <c r="D19" s="3" t="s">
-        <v>9</v>
-      </c>
-      <c r="E19" s="3" t="s">
-        <v>9</v>
-      </c>
-      <c r="F19" s="3" t="s">
-        <v>9</v>
-      </c>
-      <c r="G19" s="5" t="s">
-        <v>9</v>
-      </c>
-      <c r="H19" s="3" t="s">
-        <v>9</v>
-      </c>
-      <c r="I19" s="3" t="s">
-        <v>9</v>
-      </c>
+      <c r="D19" s="6"/>
+      <c r="E19" s="6"/>
+      <c r="F19" s="6"/>
+      <c r="G19" s="7"/>
+      <c r="H19" s="6"/>
+      <c r="I19" s="6"/>
     </row>
     <row x14ac:dyDescent="0.25" r="20" customHeight="1" ht="19.5">
-      <c r="A20" s="3" t="s">
-        <v>9</v>
-      </c>
-      <c r="B20" s="3" t="s">
-        <v>9</v>
-      </c>
+      <c r="A20" s="6"/>
+      <c r="B20" s="6"/>
       <c r="C20" s="4"/>
-      <c r="D20" s="3" t="s">
-        <v>9</v>
-      </c>
-      <c r="E20" s="3" t="s">
-        <v>9</v>
-      </c>
-      <c r="F20" s="3" t="s">
-        <v>9</v>
-      </c>
-      <c r="G20" s="5" t="s">
-        <v>9</v>
-      </c>
-      <c r="H20" s="3" t="s">
-        <v>9</v>
-      </c>
-      <c r="I20" s="3" t="s">
-        <v>9</v>
-      </c>
+      <c r="D20" s="6"/>
+      <c r="E20" s="6"/>
+      <c r="F20" s="6"/>
+      <c r="G20" s="7"/>
+      <c r="H20" s="6"/>
+      <c r="I20" s="6"/>
     </row>
     <row x14ac:dyDescent="0.25" r="21" customHeight="1" ht="19.5">
-      <c r="A21" s="3" t="s">
-        <v>9</v>
-      </c>
-      <c r="B21" s="3" t="s">
-        <v>9</v>
-      </c>
+      <c r="A21" s="6"/>
+      <c r="B21" s="6"/>
       <c r="C21" s="4"/>
-      <c r="D21" s="3" t="s">
-        <v>9</v>
-      </c>
-      <c r="E21" s="3" t="s">
-        <v>9</v>
-      </c>
-      <c r="F21" s="3" t="s">
-        <v>9</v>
-      </c>
-      <c r="G21" s="5" t="s">
-        <v>9</v>
-      </c>
-      <c r="H21" s="3" t="s">
-        <v>9</v>
-      </c>
-      <c r="I21" s="3" t="s">
-        <v>9</v>
-      </c>
+      <c r="D21" s="6"/>
+      <c r="E21" s="6"/>
+      <c r="F21" s="6"/>
+      <c r="G21" s="7"/>
+      <c r="H21" s="6"/>
+      <c r="I21" s="6"/>
     </row>
     <row x14ac:dyDescent="0.25" r="22" customHeight="1" ht="19.5">
-      <c r="A22" s="3" t="s">
-        <v>9</v>
-      </c>
-      <c r="B22" s="3" t="s">
-        <v>9</v>
-      </c>
+      <c r="A22" s="6"/>
+      <c r="B22" s="6"/>
       <c r="C22" s="4"/>
-      <c r="D22" s="3" t="s">
-        <v>9</v>
-      </c>
-      <c r="E22" s="3" t="s">
-        <v>9</v>
-      </c>
-      <c r="F22" s="3" t="s">
-        <v>9</v>
-      </c>
-      <c r="G22" s="5" t="s">
-        <v>9</v>
-      </c>
-      <c r="H22" s="3" t="s">
-        <v>9</v>
-      </c>
-      <c r="I22" s="3" t="s">
-        <v>9</v>
-      </c>
+      <c r="D22" s="6"/>
+      <c r="E22" s="6"/>
+      <c r="F22" s="6"/>
+      <c r="G22" s="7"/>
+      <c r="H22" s="6"/>
+      <c r="I22" s="6"/>
     </row>
     <row x14ac:dyDescent="0.25" r="23" customHeight="1" ht="19.5">
-      <c r="A23" s="3" t="s">
-        <v>9</v>
-      </c>
-      <c r="B23" s="3" t="s">
-        <v>9</v>
-      </c>
+      <c r="A23" s="6"/>
+      <c r="B23" s="6"/>
       <c r="C23" s="4"/>
-      <c r="D23" s="3" t="s">
-        <v>9</v>
-      </c>
-      <c r="E23" s="3" t="s">
-        <v>9</v>
-      </c>
-      <c r="F23" s="3" t="s">
-        <v>9</v>
-      </c>
-      <c r="G23" s="5" t="s">
-        <v>9</v>
-      </c>
-      <c r="H23" s="3" t="s">
-        <v>9</v>
-      </c>
-      <c r="I23" s="3" t="s">
-        <v>9</v>
-      </c>
+      <c r="D23" s="6"/>
+      <c r="E23" s="6"/>
+      <c r="F23" s="6"/>
+      <c r="G23" s="7"/>
+      <c r="H23" s="6"/>
+      <c r="I23" s="6"/>
     </row>
     <row x14ac:dyDescent="0.25" r="24" customHeight="1" ht="17.25">
-      <c r="A24" s="3" t="s">
-        <v>9</v>
-      </c>
-      <c r="B24" s="3" t="s">
-        <v>9</v>
-      </c>
+      <c r="A24" s="6"/>
+      <c r="B24" s="6"/>
       <c r="C24" s="4"/>
-      <c r="D24" s="3" t="s">
-        <v>9</v>
-      </c>
-      <c r="E24" s="3" t="s">
-        <v>9</v>
-      </c>
-      <c r="F24" s="3" t="s">
-        <v>9</v>
-      </c>
-      <c r="G24" s="5" t="s">
-        <v>9</v>
-      </c>
-      <c r="H24" s="3" t="s">
-        <v>9</v>
-      </c>
-      <c r="I24" s="3" t="s">
-        <v>9</v>
-      </c>
+      <c r="D24" s="6"/>
+      <c r="E24" s="6"/>
+      <c r="F24" s="6"/>
+      <c r="G24" s="7"/>
+      <c r="H24" s="6"/>
+      <c r="I24" s="6"/>
     </row>
     <row x14ac:dyDescent="0.25" r="25" customHeight="1" ht="17.25">
-      <c r="A25" s="3" t="s">
-        <v>9</v>
-      </c>
-      <c r="B25" s="3" t="s">
-        <v>9</v>
-      </c>
+      <c r="A25" s="6"/>
+      <c r="B25" s="6"/>
       <c r="C25" s="4"/>
-      <c r="D25" s="3" t="s">
-        <v>9</v>
-      </c>
-      <c r="E25" s="3" t="s">
-        <v>9</v>
-      </c>
-      <c r="F25" s="3" t="s">
-        <v>9</v>
-      </c>
-      <c r="G25" s="5" t="s">
-        <v>9</v>
-      </c>
-      <c r="H25" s="3" t="s">
-        <v>9</v>
-      </c>
-      <c r="I25" s="3" t="s">
-        <v>9</v>
-      </c>
+      <c r="D25" s="6"/>
+      <c r="E25" s="6"/>
+      <c r="F25" s="6"/>
+      <c r="G25" s="7"/>
+      <c r="H25" s="6"/>
+      <c r="I25" s="6"/>
     </row>
     <row x14ac:dyDescent="0.25" r="26" customHeight="1" ht="17.25">
-      <c r="A26" s="3" t="s">
-        <v>9</v>
-      </c>
-      <c r="B26" s="3" t="s">
-        <v>9</v>
-      </c>
+      <c r="A26" s="6"/>
+      <c r="B26" s="6"/>
       <c r="C26" s="4"/>
-      <c r="D26" s="3" t="s">
-        <v>9</v>
-      </c>
-      <c r="E26" s="3" t="s">
-        <v>9</v>
-      </c>
-      <c r="F26" s="3" t="s">
-        <v>9</v>
-      </c>
-      <c r="G26" s="5" t="s">
-        <v>9</v>
-      </c>
-      <c r="H26" s="3" t="s">
-        <v>9</v>
-      </c>
-      <c r="I26" s="3" t="s">
-        <v>9</v>
-      </c>
+      <c r="D26" s="6"/>
+      <c r="E26" s="6"/>
+      <c r="F26" s="6"/>
+      <c r="G26" s="7"/>
+      <c r="H26" s="6"/>
+      <c r="I26" s="6"/>
     </row>
     <row x14ac:dyDescent="0.25" r="27" customHeight="1" ht="17.25">
-      <c r="A27" s="3" t="s">
-        <v>9</v>
-      </c>
-      <c r="B27" s="3" t="s">
-        <v>9</v>
-      </c>
+      <c r="A27" s="6"/>
+      <c r="B27" s="6"/>
       <c r="C27" s="4"/>
-      <c r="D27" s="3" t="s">
-        <v>9</v>
-      </c>
-      <c r="E27" s="3" t="s">
-        <v>9</v>
-      </c>
-      <c r="F27" s="3" t="s">
-        <v>9</v>
-      </c>
-      <c r="G27" s="5" t="s">
-        <v>9</v>
-      </c>
-      <c r="H27" s="3" t="s">
-        <v>9</v>
-      </c>
-      <c r="I27" s="3" t="s">
-        <v>9</v>
-      </c>
+      <c r="D27" s="6"/>
+      <c r="E27" s="6"/>
+      <c r="F27" s="6"/>
+      <c r="G27" s="7"/>
+      <c r="H27" s="6"/>
+      <c r="I27" s="6"/>
     </row>
     <row x14ac:dyDescent="0.25" r="28" customHeight="1" ht="17.25">
-      <c r="A28" s="3" t="s">
-        <v>9</v>
-      </c>
-      <c r="B28" s="3" t="s">
-        <v>9</v>
-      </c>
+      <c r="A28" s="6"/>
+      <c r="B28" s="6"/>
       <c r="C28" s="4"/>
-      <c r="D28" s="3" t="s">
-        <v>9</v>
-      </c>
-      <c r="E28" s="3" t="s">
-        <v>9</v>
-      </c>
-      <c r="F28" s="3" t="s">
-        <v>9</v>
-      </c>
-      <c r="G28" s="5" t="s">
-        <v>9</v>
-      </c>
-      <c r="H28" s="3" t="s">
-        <v>9</v>
-      </c>
-      <c r="I28" s="3" t="s">
-        <v>9</v>
-      </c>
+      <c r="D28" s="6"/>
+      <c r="E28" s="6"/>
+      <c r="F28" s="6"/>
+      <c r="G28" s="7"/>
+      <c r="H28" s="6"/>
+      <c r="I28" s="6"/>
     </row>
     <row x14ac:dyDescent="0.25" r="29" customHeight="1" ht="17.25">
-      <c r="A29" s="3" t="s">
-        <v>9</v>
-      </c>
-      <c r="B29" s="3" t="s">
-        <v>9</v>
-      </c>
+      <c r="A29" s="6"/>
+      <c r="B29" s="6"/>
       <c r="C29" s="4"/>
-      <c r="D29" s="3" t="s">
-        <v>9</v>
-      </c>
-      <c r="E29" s="3" t="s">
-        <v>9</v>
-      </c>
-      <c r="F29" s="3" t="s">
-        <v>9</v>
-      </c>
-      <c r="G29" s="5" t="s">
-        <v>9</v>
-      </c>
-      <c r="H29" s="3" t="s">
-        <v>9</v>
-      </c>
-      <c r="I29" s="3" t="s">
-        <v>9</v>
-      </c>
+      <c r="D29" s="6"/>
+      <c r="E29" s="6"/>
+      <c r="F29" s="6"/>
+      <c r="G29" s="7"/>
+      <c r="H29" s="6"/>
+      <c r="I29" s="6"/>
     </row>
     <row x14ac:dyDescent="0.25" r="30" customHeight="1" ht="17.25">
-      <c r="A30" s="3" t="s">
-        <v>9</v>
-      </c>
-      <c r="B30" s="3" t="s">
-        <v>9</v>
-      </c>
-      <c r="C30" s="6"/>
-      <c r="D30" s="3" t="s">
-        <v>9</v>
-      </c>
-      <c r="E30" s="3" t="s">
-        <v>9</v>
-      </c>
-      <c r="F30" s="3" t="s">
-        <v>9</v>
-      </c>
-      <c r="G30" s="5" t="s">
-        <v>9</v>
-      </c>
-      <c r="H30" s="3" t="s">
-        <v>9</v>
-      </c>
-      <c r="I30" s="3" t="s">
-        <v>9</v>
-      </c>
+      <c r="A30" s="6"/>
+      <c r="B30" s="6"/>
+      <c r="C30" s="4"/>
+      <c r="D30" s="6"/>
+      <c r="E30" s="6"/>
+      <c r="F30" s="6"/>
+      <c r="G30" s="7"/>
+      <c r="H30" s="6"/>
+      <c r="I30" s="6"/>
     </row>
     <row x14ac:dyDescent="0.25" r="31" customHeight="1" ht="17.25">
-      <c r="A31" s="3" t="s">
-        <v>9</v>
-      </c>
-      <c r="B31" s="3" t="s">
-        <v>9</v>
-      </c>
-      <c r="C31" s="6"/>
-      <c r="D31" s="3" t="s">
-        <v>9</v>
-      </c>
-      <c r="E31" s="3" t="s">
-        <v>9</v>
-      </c>
-      <c r="F31" s="3" t="s">
-        <v>9</v>
-      </c>
-      <c r="G31" s="7" t="s">
-        <v>9</v>
-      </c>
-      <c r="H31" s="3" t="s">
-        <v>9</v>
-      </c>
-      <c r="I31" s="3" t="s">
-        <v>9</v>
-      </c>
+      <c r="A31" s="6"/>
+      <c r="B31" s="6"/>
+      <c r="C31" s="4"/>
+      <c r="D31" s="6"/>
+      <c r="E31" s="6"/>
+      <c r="F31" s="6"/>
+      <c r="G31" s="8"/>
+      <c r="H31" s="6"/>
+      <c r="I31" s="6"/>
     </row>
     <row x14ac:dyDescent="0.25" r="32" customHeight="1" ht="17.25">
-      <c r="A32" s="3" t="s">
-        <v>9</v>
-      </c>
-      <c r="B32" s="3" t="s">
-        <v>9</v>
-      </c>
-      <c r="C32" s="6"/>
-      <c r="D32" s="3" t="s">
-        <v>9</v>
-      </c>
-      <c r="E32" s="3" t="s">
-        <v>9</v>
-      </c>
-      <c r="F32" s="3" t="s">
-        <v>9</v>
-      </c>
-      <c r="G32" s="7" t="s">
-        <v>9</v>
-      </c>
-      <c r="H32" s="3" t="s">
-        <v>9</v>
-      </c>
-      <c r="I32" s="3" t="s">
-        <v>9</v>
-      </c>
+      <c r="A32" s="6"/>
+      <c r="B32" s="6"/>
+      <c r="C32" s="4"/>
+      <c r="D32" s="6"/>
+      <c r="E32" s="6"/>
+      <c r="F32" s="6"/>
+      <c r="G32" s="8"/>
+      <c r="H32" s="6"/>
+      <c r="I32" s="6"/>
     </row>
     <row x14ac:dyDescent="0.25" r="33" customHeight="1" ht="17.25">
-      <c r="A33" s="3" t="s">
-        <v>9</v>
-      </c>
-      <c r="B33" s="3" t="s">
-        <v>9</v>
-      </c>
-      <c r="C33" s="6"/>
-      <c r="D33" s="3" t="s">
-        <v>9</v>
-      </c>
-      <c r="E33" s="3" t="s">
-        <v>9</v>
-      </c>
-      <c r="F33" s="3" t="s">
-        <v>9</v>
-      </c>
-      <c r="G33" s="5" t="s">
-        <v>9</v>
-      </c>
-      <c r="H33" s="3" t="s">
-        <v>9</v>
-      </c>
-      <c r="I33" s="3" t="s">
-        <v>9</v>
-      </c>
+      <c r="A33" s="6"/>
+      <c r="B33" s="6"/>
+      <c r="C33" s="4"/>
+      <c r="D33" s="6"/>
+      <c r="E33" s="6"/>
+      <c r="F33" s="6"/>
+      <c r="G33" s="7"/>
+      <c r="H33" s="6"/>
+      <c r="I33" s="6"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>